<commit_message>
Prototype data cleanup prepared
</commit_message>
<xml_diff>
--- a/src/ex.xlsx
+++ b/src/ex.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,57 +446,52 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>supported_languages</t>
+          <t>developers</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>developers</t>
+          <t>publishers</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>publishers</t>
+          <t>price_overview</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>price_overview</t>
+          <t>categories</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>categories</t>
+          <t>genres</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>genres</t>
+          <t>recommendations</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>achievements</t>
+          <t>controller_support</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>release_date</t>
+          <t>dlc_count</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>dlc</t>
+          <t>achievements_count</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>recommendations</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>controller_support</t>
+          <t>release_year</t>
         </is>
       </c>
     </row>
@@ -519,7 +514,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>EckGames</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -527,44 +522,35 @@
           <t>EckGames</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>EckGames</t>
-        </is>
+      <c r="G2" t="n">
+        <v>899</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PLN 899 899</t>
+          <t>Single-player, Steam Achievements, Steam Cloud, Steam Leaderboards, Family Sharing</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Steam Cloud, Steam Leaderboards, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
           <t>Action, Adventure, Casual, Indie</t>
         </is>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0 06/02/2018</t>
-        </is>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="3">
@@ -586,7 +572,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , Korean, Traditional Chinese, Simplified Chinese     </t>
+          <t>Masangsoft</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -594,40 +580,35 @@
           <t>Masangsoft</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Masangsoft</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Multi-player, MMO, PvP, Online PvP, Co-op, Online Co-op, Steam Achievements, In-App Purchases</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Multi-player, MMO, PvP, Online PvP, Co-op, Online Co-op, Steam Achievements, In-App Purchases</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
           <t>Action, Adventure, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0 05/03/2019</t>
-        </is>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>5</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2019</v>
       </c>
     </row>
     <row r="4">
@@ -653,7 +634,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , Traditional Chinese, Ukrainian     </t>
+          <t>Holomia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -661,40 +642,35 @@
           <t>Holomia</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Holomia</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Single-player, Multi-player, PvP, LAN PvP, Co-op, LAN Co-op, Cross-Platform Multiplayer</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Single-player, Multi-player, PvP, LAN PvP, Co-op, LAN Co-op, Cross-Platform Multiplayer</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
           <t>Action, Simulation</t>
         </is>
       </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0 20/07/2018</t>
-        </is>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="5">
@@ -716,7 +692,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>English, Japanese</t>
+          <t>Chilla's Art</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -724,44 +700,35 @@
           <t>Chilla's Art</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Chilla's Art</t>
-        </is>
+      <c r="G5" t="n">
+        <v>1349</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PLN 1349 1349</t>
+          <t>Single-player, Partial Controller Support, Family Sharing</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Single-player, Partial Controller Support, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
           <t>Adventure, Casual, Indie</t>
         </is>
       </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>0 15/02/2018</t>
-        </is>
+      <c r="J5" t="n">
+        <v>163</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>163</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="6">
@@ -798,52 +765,43 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>CSM</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CSM</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
           <t>W.T.B.</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>2299</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PLN 2299 2299</t>
+          <t>Single-player, Steam Achievements, Family Sharing</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
           <t>Casual, Indie</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>1</v>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>0 22/01/2018</t>
-        </is>
-      </c>
       <c r="M6" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="7">
@@ -865,7 +823,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Penumbra Games</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -873,44 +831,35 @@
           <t>Penumbra Games</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Penumbra Games</t>
-        </is>
+      <c r="G7" t="n">
+        <v>719</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PLN 719 719</t>
+          <t>Single-player, Steam Achievements, Steam Cloud, Family Sharing</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Steam Cloud, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
           <t>Violent, Gore, Adventure, Indie</t>
         </is>
       </c>
-      <c r="K7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>0 26/01/2018</t>
-        </is>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="8">
@@ -932,7 +881,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>English, Spanish - Spain, Polish, French, Italian, German, Simplified Chinese, Japanese, Korean, Portuguese - Brazil, Turkish</t>
+          <t>Koksny.com</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -940,44 +889,35 @@
           <t>Koksny.com</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Koksny.com</t>
-        </is>
+      <c r="G8" t="n">
+        <v>5399</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PLN 5399 5399</t>
+          <t>Single-player, Steam Achievements, Steam Workshop, Partial Controller Support, Steam Cloud, Stats, Includes level editor, Family Sharing</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Steam Workshop, Partial Controller Support, Steam Cloud, Stats, Includes level editor, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
           <t>Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="K8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>0 31/03/2021</t>
-        </is>
+      <c r="J8" t="n">
+        <v>214</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="N8" t="n">
-        <v>214</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2021</v>
       </c>
     </row>
     <row r="9">
@@ -999,52 +939,43 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , French, German, Spanish - Spain, Russian, Polish, Simplified Chinese     </t>
+          <t>Osaris Games</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Osaris Games</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
           <t>RockGame S.A.</t>
         </is>
       </c>
+      <c r="G9" t="n">
+        <v>6499</v>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>PLN 6499 6499</t>
+          <t>Single-player, Multi-player, Co-op, Online Co-op, Steam Achievements, Steam Workshop, Family Sharing</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Single-player, Multi-player, Co-op, Online Co-op, Steam Achievements, Steam Workshop, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
           <t>Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="K9" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>0 15/09/2022</t>
-        </is>
+      <c r="J9" t="n">
+        <v>192</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="N9" t="n">
-        <v>192</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2022</v>
       </c>
     </row>
     <row r="10">
@@ -1066,7 +997,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>English, Japanese, Korean, Simplified Chinese, Russian</t>
+          <t>narayana games UG</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1074,41 +1005,34 @@
           <t>narayana games UG</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>narayana games UG</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Single-player, Multi-player, Co-op, Online Co-op, LAN Co-op, Shared/Split Screen Co-op, Shared/Split Screen, Cross-Platform Multiplayer, Steam Achievements, Tracked Controller Support, VR Only, In-App Purchases, Stats, Steam Leaderboards, Includes level editor, Family Sharing</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Single-player, Multi-player, Co-op, Online Co-op, LAN Co-op, Shared/Split Screen Co-op, Shared/Split Screen, Cross-Platform Multiplayer, Steam Achievements, Tracked Controller Support, VR Only, In-App Purchases, Stats, Steam Leaderboards, Includes level editor, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
           <t>Casual, Indie, Sports</t>
         </is>
       </c>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>1 To be announced</t>
-        </is>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1131,52 +1055,43 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Infogrames</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Infogrames</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
           <t>Atari</t>
         </is>
       </c>
+      <c r="G11" t="n">
+        <v>2899</v>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>PLN 2899 2899</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
           <t>Adventure, RPG</t>
         </is>
       </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>0 08/02/2018</t>
-        </is>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="12">
@@ -1205,52 +1120,43 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Infogrames</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Infogrames</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
           <t xml:space="preserve">Ziggurat </t>
         </is>
       </c>
+      <c r="G12" t="n">
+        <v>1799</v>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>PLN 1799 539</t>
+          <t>Single-player, Multi-player, PvP, Shared/Split Screen PvP, Co-op, Remote Play Together, Family Sharing</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Single-player, Multi-player, PvP, Shared/Split Screen PvP, Co-op, Remote Play Together, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="K12" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>0 08/02/2018</t>
-        </is>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="13">
@@ -1280,52 +1186,43 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Infogrames</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Infogrames</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
           <t>Ziggurat</t>
         </is>
       </c>
+      <c r="G13" t="n">
+        <v>2549</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>PLN 2549 2549</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
           <t>Action, Adventure</t>
         </is>
       </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>0 08/02/2018</t>
-        </is>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="14">
@@ -1359,52 +1256,43 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Infogrames</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Infogrames</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
           <t>Ziggurat</t>
         </is>
       </c>
+      <c r="G14" t="n">
+        <v>2549</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>PLN 2549 764</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
           <t>Action, Adventure, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="K14" t="n">
-        <v>1</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>0 08/02/2018</t>
-        </is>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="15">
@@ -1437,52 +1325,43 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Infogrames</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Infogrames</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
           <t>Ziggurat</t>
         </is>
       </c>
+      <c r="G15" t="n">
+        <v>2549</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>PLN 2549 764</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
           <t>Action, Adventure</t>
         </is>
       </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>0 08/02/2018</t>
-        </is>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="16">
@@ -1523,52 +1402,43 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Infogrames</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Infogrames</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
           <t>Ziggurat</t>
         </is>
       </c>
+      <c r="G16" t="n">
+        <v>2549</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>PLN 2549 2549</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
           <t>Action, Adventure, RPG</t>
         </is>
       </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>0 08/02/2018</t>
-        </is>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="17">
@@ -1606,52 +1476,43 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Infogrames</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Infogrames</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
           <t>Atari</t>
         </is>
       </c>
+      <c r="G17" t="n">
+        <v>2549</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>PLN 2549 2549</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
           <t>Action, Strategy</t>
         </is>
       </c>
-      <c r="K17" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>0 08/02/2018</t>
-        </is>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="18">
@@ -1673,7 +1534,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>VR Factory</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1681,44 +1542,35 @@
           <t>VR Factory</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>VR Factory</t>
-        </is>
+      <c r="G18" t="n">
+        <v>3599</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>PLN 3599 3599</t>
+          <t>Single-player, Tracked Controller Support, VR Only, Family Sharing</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Single-player, Tracked Controller Support, VR Only, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
           <t>Action, Casual, Indie</t>
         </is>
       </c>
-      <c r="K18" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>0 26/01/2018</t>
-        </is>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="19">
@@ -1740,48 +1592,43 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , Russian        </t>
+          <t>Foxoft</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Foxoft</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
           <t>AZAMATIKA</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Single-player, Steam Achievements, Full controller support</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Full controller support</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
           <t>Action, Adventure, Indie</t>
         </is>
       </c>
-      <c r="K19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>0 20/02/2018</t>
-        </is>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="20">
@@ -1803,52 +1650,43 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Ethan Summers Alex Lamb Nainoa Faulkner-Jackson Lauren Hanf Ramsey Antrim-Kerr Kieran Wright Anne-Marie Napoli</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Ethan Summers Alex Lamb Nainoa Faulkner-Jackson Lauren Hanf Ramsey Antrim-Kerr Kieran Wright Anne-Marie Napoli</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
           <t>Almost Human Media</t>
         </is>
       </c>
+      <c r="G20" t="n">
+        <v>8299</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>PLN 8299 8299</t>
+          <t>Single-player, VR Supported, Family Sharing</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Single-player, VR Supported, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
           <t>Casual, Indie</t>
         </is>
       </c>
-      <c r="K20" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>0 14/11/2024</t>
-        </is>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2024</v>
       </c>
     </row>
     <row r="21">
@@ -1870,52 +1708,43 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>English, German, Simplified Chinese</t>
+          <t>Dragon Slumber</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Dragon Slumber</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
           <t>Iceberg Interactive</t>
         </is>
       </c>
+      <c r="G21" t="n">
+        <v>4599</v>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>PLN 4599 4599</t>
+          <t>Single-player, Steam Achievements, Steam Trading Cards, Steam Cloud, Family Sharing</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Steam Trading Cards, Steam Cloud, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
           <t>Adventure, Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="K21" t="n">
-        <v>1</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>0 27/02/2019</t>
-        </is>
+      <c r="J21" t="n">
+        <v>561</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="N21" t="n">
-        <v>561</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2019</v>
       </c>
     </row>
     <row r="22">
@@ -1937,7 +1766,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>English, Simplified Chinese, Traditional Chinese</t>
+          <t>Fish Chain Games</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1945,44 +1774,35 @@
           <t>Fish Chain Games</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Fish Chain Games</t>
-        </is>
+      <c r="G22" t="n">
+        <v>899</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>PLN 899 899</t>
+          <t>Single-player, Steam Achievements, Full controller support, Steam Cloud, Stats, Family Sharing</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Full controller support, Steam Cloud, Stats, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
           <t>Casual, Indie</t>
         </is>
       </c>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>0 05/02/2018</t>
-        </is>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="23">
@@ -2004,7 +1824,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , Simplified Chinese   , Traditional Chinese        </t>
+          <t>BD Studio Games</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2012,44 +1832,35 @@
           <t>BD Studio Games</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>BD Studio Games</t>
-        </is>
+      <c r="G23" t="n">
+        <v>1099</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>PLN 1099 1099</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
           <t>Action, Casual, Indie</t>
         </is>
       </c>
-      <c r="K23" t="n">
-        <v>1</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>0 31/01/2018</t>
-        </is>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="24">
@@ -2071,7 +1882,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Eternity Studios</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2079,44 +1890,35 @@
           <t>Eternity Studios</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Eternity Studios</t>
-        </is>
+      <c r="G24" t="n">
+        <v>1449</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>PLN 1449 1449</t>
+          <t>Single-player, Steam Achievements, Family Sharing</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
           <t>Action, Adventure, Casual, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="K24" t="n">
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
         <v>1</v>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>0 28/01/2018</t>
-        </is>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="25">
@@ -2138,7 +1940,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Simplified Chinese   , Traditional Chinese        </t>
+          <t>Flying Star Games</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2146,44 +1948,35 @@
           <t>Flying Star Games</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Flying Star Games</t>
-        </is>
+      <c r="G25" t="n">
+        <v>2199</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>PLN 2199 2199</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
           <t>Adventure, RPG, Strategy</t>
         </is>
       </c>
-      <c r="K25" t="n">
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
         <v>1</v>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>0 02/02/2018</t>
-        </is>
-      </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="26">
@@ -2212,52 +2005,43 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>ARGames</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ARGames</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
           <t>Metal Fox</t>
         </is>
       </c>
+      <c r="G26" t="n">
+        <v>449</v>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>PLN 449 449</t>
+          <t>Single-player, Steam Achievements, Family Sharing</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
           <t>Adventure, Indie</t>
         </is>
       </c>
-      <c r="K26" t="n">
-        <v>1</v>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>0 24/01/2018</t>
-        </is>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="27">
@@ -2279,52 +2063,43 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Iffy Labs</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Iffy Labs</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
           <t>hOSHI</t>
         </is>
       </c>
+      <c r="G27" t="n">
+        <v>2199</v>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>PLN 2199 2199</t>
+          <t>Multi-player, PvP, Online PvP, Shared/Split Screen PvP, Co-op, Online Co-op, Shared/Split Screen Co-op, Shared/Split Screen, Steam Achievements, Full controller support, Remote Play Together, Family Sharing</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Multi-player, PvP, Online PvP, Shared/Split Screen PvP, Co-op, Online Co-op, Shared/Split Screen Co-op, Shared/Split Screen, Steam Achievements, Full controller support, Remote Play Together, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
           <t>Action, Casual, Indie, Strategy</t>
         </is>
       </c>
-      <c r="K27" t="n">
-        <v>1</v>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>0 01/02/2019</t>
-        </is>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>2019</v>
       </c>
     </row>
     <row r="28">
@@ -2346,7 +2121,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Luke O'Connor</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2354,44 +2129,35 @@
           <t>Luke O'Connor</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Luke O'Connor</t>
-        </is>
+      <c r="G28" t="n">
+        <v>2549</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>PLN 2549 2549</t>
+          <t>Single-player, Partial Controller Support, Family Sharing</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Single-player, Partial Controller Support, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
           <t>Action, Casual, Indie</t>
         </is>
       </c>
-      <c r="K28" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>0 02/05/2018</t>
-        </is>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="29">
@@ -2433,7 +2199,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>FurGoldGames</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2441,44 +2207,35 @@
           <t>FurGoldGames</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>FurGoldGames</t>
-        </is>
+      <c r="G29" t="n">
+        <v>359</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>PLN 359 359</t>
+          <t>Single-player, Steam Achievements, Steam Leaderboards, Family Sharing</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Steam Leaderboards, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
           <t>Indie, Racing, Simulation</t>
         </is>
       </c>
-      <c r="K29" t="n">
-        <v>1</v>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>0 23/01/2018</t>
-        </is>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="30">
@@ -2500,7 +2257,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>RewindApp</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2508,44 +2265,35 @@
           <t>RewindApp</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>RewindApp</t>
-        </is>
+      <c r="G30" t="n">
+        <v>800</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>PLN 800 800</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
           <t>Casual, Indie</t>
         </is>
       </c>
-      <c r="K30" t="n">
-        <v>1</v>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>0 07/02/2018</t>
-        </is>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="31">
@@ -2567,7 +2315,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Magnolia Art</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2575,40 +2323,35 @@
           <t>Magnolia Art</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Magnolia Art</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Single-player, Steam Achievements, Steam Cloud, Steam Leaderboards</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Steam Cloud, Steam Leaderboards</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
           <t>Casual, Indie</t>
         </is>
       </c>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>0 07/03/2018</t>
-        </is>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="N31" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="32">
@@ -2630,7 +2373,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>ocasocreations</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2638,44 +2381,35 @@
           <t>ocasocreations</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>ocasocreations</t>
-        </is>
+      <c r="G32" t="n">
+        <v>3699</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>PLN 3699 3699</t>
+          <t>Single-player, Multi-player, PvP, Shared/Split Screen PvP, Shared/Split Screen, Steam Achievements, Partial Controller Support, Remote Play Together, Family Sharing</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Single-player, Multi-player, PvP, Shared/Split Screen PvP, Shared/Split Screen, Steam Achievements, Partial Controller Support, Remote Play Together, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
           <t>Indie</t>
         </is>
       </c>
-      <c r="K32" t="n">
-        <v>1</v>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>0 18/03/2019</t>
-        </is>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="N32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2019</v>
       </c>
     </row>
     <row r="33">
@@ -2705,7 +2439,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Sick Kreations</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2713,41 +2447,34 @@
           <t>Sick Kreations</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Sick Kreations</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Multi-player, PvP, Online PvP, Family Sharing</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Multi-player, PvP, Online PvP, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="K33" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>1 Coming soon</t>
-        </is>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -2776,7 +2503,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Ripknot Systems</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2784,44 +2511,35 @@
           <t>Ripknot Systems</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Ripknot Systems</t>
-        </is>
+      <c r="G34" t="n">
+        <v>6399</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>PLN 6399 6399</t>
+          <t>Single-player, Steam Achievements, Family Sharing</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
           <t>Casual, Indie, Simulation, Strategy</t>
         </is>
       </c>
-      <c r="K34" t="n">
-        <v>1</v>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>0 23/01/2018</t>
-        </is>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="35">
@@ -2843,7 +2561,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>AnderShi</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2851,44 +2569,35 @@
           <t>AnderShi</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>AnderShi</t>
-        </is>
+      <c r="G35" t="n">
+        <v>359</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>PLN 359 359</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
           <t>Adventure, Indie, Simulation</t>
         </is>
       </c>
-      <c r="K35" t="n">
-        <v>1</v>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>0 03/05/2018</t>
-        </is>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="36">
@@ -2910,7 +2619,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Sigil Softworks</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2918,41 +2627,34 @@
           <t>Sigil Softworks</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Sigil Softworks</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Multi-player, PvP, Online PvP, Co-op, Online Co-op, Steam Achievements, Full controller support, Family Sharing</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Multi-player, PvP, Online PvP, Co-op, Online Co-op, Steam Achievements, Full controller support, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="K36" t="n">
-        <v>1</v>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>1 To be announced</t>
-        </is>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
-      </c>
-      <c r="N36" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -2973,52 +2675,43 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>English, Russian</t>
+          <t>TheDreik Xeneder</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>TheDreik Xeneder</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
           <t>Phoenix Reborn Games</t>
         </is>
       </c>
+      <c r="G37" t="n">
+        <v>449</v>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>PLN 449 449</t>
+          <t>Single-player, Steam Achievements, Full controller support, Family Sharing</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Full controller support, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="K37" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>0 26/01/2018</t>
-        </is>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="N37" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="38">
@@ -3040,7 +2733,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , French   , Italian   , German   , Spanish - Spain   , Arabic   , Bulgarian   , Portuguese - Brazil   , Hungarian   , Greek   , Danish   , Traditional Chinese   , Simplified Chinese   , Korean   , Dutch   , Norwegian   , Polish   , Portuguese - Portugal   , Romanian   , Russian   , Thai   , Turkish   , Ukrainian   , Finnish   , Czech   , Swedish   , Japanese   , Vietnamese   , Spanish - Latin America        </t>
+          <t>Crew Lab</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3048,44 +2741,35 @@
           <t>Crew Lab</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Crew Lab</t>
-        </is>
+      <c r="G38" t="n">
+        <v>449</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>PLN 449 449</t>
+          <t>Single-player, Steam Achievements, Family Sharing</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
           <t>Casual, Indie</t>
         </is>
       </c>
-      <c r="K38" t="n">
+      <c r="J38" t="n">
+        <v>325</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
         <v>1</v>
       </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>0 17/06/2018</t>
-        </is>
-      </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>1800</v>
       </c>
       <c r="N38" t="n">
-        <v>325</v>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="39">
@@ -3107,7 +2791,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , French   , Italian   , German   , Spanish - Spain   , Arabic   , Bulgarian   , Portuguese - Brazil   , Hungarian   , Greek   , Danish   , Traditional Chinese   , Simplified Chinese   , Korean   , Dutch   , Norwegian   , Polish   , Portuguese - Portugal   , Romanian   , Russian   , Thai   , Turkish   , Ukrainian   , Finnish   , Czech   , Swedish   , Japanese   , Vietnamese   , Spanish - Latin America        </t>
+          <t>Crew Lab</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3115,44 +2799,35 @@
           <t>Crew Lab</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Crew Lab</t>
-        </is>
+      <c r="G39" t="n">
+        <v>449</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>PLN 449 449</t>
+          <t>Single-player, Steam Achievements, Family Sharing</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
           <t>Casual, Indie</t>
         </is>
       </c>
-      <c r="K39" t="n">
+      <c r="J39" t="n">
+        <v>220</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
         <v>1</v>
       </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>0 31/05/2018</t>
-        </is>
-      </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>2230</v>
       </c>
       <c r="N39" t="n">
-        <v>220</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="40">
@@ -3174,7 +2849,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>90E GAMES</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3182,44 +2857,35 @@
           <t>90E GAMES</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>90E GAMES</t>
-        </is>
+      <c r="G40" t="n">
+        <v>449</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>PLN 449 449</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
           <t>Action, Adventure, Casual, Indie, Simulation</t>
         </is>
       </c>
-      <c r="K40" t="n">
-        <v>1</v>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>0 31/01/2018</t>
-        </is>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="41">
@@ -3241,7 +2907,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">English   , German, Spanish - Spain, Spanish - Latin America, Portuguese - Brazil, Portuguese - Portugal, Polish     </t>
+          <t>Crystal Shard</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3249,44 +2915,35 @@
           <t>Crystal Shard</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Crystal Shard</t>
-        </is>
+      <c r="G41" t="n">
+        <v>4599</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>PLN 4599 4599</t>
+          <t>Single-player, Steam Achievements, Full controller support, Steam Workshop, Camera Comfort, Color Alternatives, Custom Volume Controls, Adjustable Difficulty, Keyboard Only Option, Playable without Timed Input, Subtitle Options, Steam Cloud, Steam Leaderboards, Includes level editor, Family Sharing</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Single-player, Steam Achievements, Full controller support, Steam Workshop, Camera Comfort, Color Alternatives, Custom Volume Controls, Adjustable Difficulty, Keyboard Only Option, Playable without Timed Input, Subtitle Options, Steam Cloud, Steam Leaderboards, Includes level editor, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
           <t>Action, Indie</t>
         </is>
       </c>
-      <c r="K41" t="n">
-        <v>1</v>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>0 08/12/2019</t>
-        </is>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>3</v>
       </c>
       <c r="M41" t="n">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="N41" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>2019</v>
       </c>
     </row>
     <row r="42">
@@ -3308,7 +2965,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Renegade Games</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3316,44 +2973,35 @@
           <t>Renegade Games</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Renegade Games</t>
-        </is>
+      <c r="G42" t="n">
+        <v>497</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>PLN 497 497</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
           <t>Action, Adventure, Casual, Indie</t>
         </is>
       </c>
-      <c r="K42" t="n">
-        <v>1</v>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>0 28/01/2018</t>
-        </is>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
       </c>
     </row>
     <row r="43">
@@ -3379,52 +3027,111 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">English        </t>
+          <t>Primitive Studio</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Primitive Studio</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
           <t>Conglomerate 5</t>
         </is>
       </c>
+      <c r="G43" t="n">
+        <v>449</v>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>PLN 449 449</t>
+          <t>Single-player, Family Sharing</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Single-player, Family Sharing</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
           <t>Action, Adventure, Indie, Strategy</t>
         </is>
       </c>
-      <c r="K43" t="n">
-        <v>1</v>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>0 01/02/2018</t>
-        </is>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Ball of Wonder</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Clowns are freak you out? It's time to revenge! + Ball of Wonder is an arkanoid style game, in the magnicifent world of circuses. Play througth 50 levels in 9 game mode alone or in cooperate with your friend. Destroy the puzzle elements, Ferris wheel' steats and clowns. + Ball of Wonder has 9 different power-ups and you need to activate them manualy. If you have some power-up at the and of the level, you will got them in the next one. + Remember, there is 9 different game mode in Ball of Wonder, like: + -Destroy everything + -Gather points + -Pop up the balloons + -Destroy everything in the dark + -etc +  + Oh, and before i forgot: there's two boss fight too...one of them is againts a big, bad clown. Go and catch it!</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>White Rabbit Games</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>My Way Games</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>4599</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Single-player, Multi-player, Co-op, Shared/Split Screen Co-op, Shared/Split Screen, Steam Achievements, Steam Trading Cards, Partial Controller Support, Remote Play Together, Family Sharing</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Casual, Indie</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="n">
+        <v>36</v>
+      </c>
+      <c r="N44" t="n">
+        <v>2016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>